<commit_message>
docs: enhance EDA course content by revising the Cowork section for clarity, updating practical examples, and improving session descriptions, while removing outdated files to streamline the learning experience
</commit_message>
<xml_diff>
--- a/eda/example/cowork-excel/費用報銷表.xlsx
+++ b/eda/example/cowork-excel/費用報銷表.xlsx
@@ -1,109 +1,80 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lindingyuan/Documents/external_project/agent-skills/course/eda/example/cowork-excel/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3D43C92-EC1F-6A43-A1E1-6951F9194855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="填寫說明" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="費用報銷表" state="visible" r:id="rId5"/>
+    <sheet name="費用報銷表" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
-  <si>
-    <t>差旅費用報銷表 — 填寫說明</t>
-  </si>
-  <si>
-    <t>用途</t>
-  </si>
-  <si>
-    <t>把一疊收據／單據照片，整理成可報帳的明細</t>
-  </si>
-  <si>
-    <t>欄位</t>
-  </si>
-  <si>
-    <t>規則</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>日期</t>
-  </si>
-  <si>
-    <t>收據上的消費日期，格式 YYYY-MM-DD</t>
   </si>
   <si>
     <t>費用類別</t>
   </si>
   <si>
-    <t>只能填：交通 / 住宿 / 餐費 / 其他</t>
-  </si>
-  <si>
     <t>項目說明</t>
-  </si>
-  <si>
-    <t>收據上的店家或品名（例：台灣高鐵 台北-台中）</t>
   </si>
   <si>
     <t>金額(NT$)</t>
   </si>
   <si>
-    <t>只填數字，不要加「元」或逗號</t>
-  </si>
-  <si>
     <t>單據號碼</t>
   </si>
   <si>
-    <t>收據／發票上的號碼；看不清楚就留空標黃</t>
-  </si>
-  <si>
     <t>備註</t>
-  </si>
-  <si>
-    <t>補充說明（例：出差會員 App 封測）</t>
-  </si>
-  <si>
-    <t>⚠️ 重要</t>
-  </si>
-  <si>
-    <t>金額一定要對得上收據；看不清楚的欄位留空標黃，不要四捨五入或猜測。整疊收據要逐張對，不漏不重。</t>
-  </si>
-  <si>
-    <t>合計</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <sz val="11"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="新細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFB00000"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -112,21 +83,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2A2A2A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF3CD"/>
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -150,29 +132,33 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -508,328 +494,248 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="24" customHeight="1">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" spans="1:7" ht="20" customHeight="1">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
       <c r="C2" s="7"/>
       <c r="D2" s="8"/>
-      <c r="E2" s="7"/>
+      <c r="E2" s="6"/>
       <c r="F2" s="7"/>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" spans="1:7" ht="20" customHeight="1">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
       <c r="C3" s="7"/>
       <c r="D3" s="8"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="6"/>
       <c r="F3" s="7"/>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" spans="1:7" ht="20" customHeight="1">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="8"/>
-      <c r="E4" s="7"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="7"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
+      <c r="G4" s="6"/>
+    </row>
+    <row r="5" spans="1:7" ht="20" customHeight="1">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
       <c r="C5" s="7"/>
       <c r="D5" s="8"/>
-      <c r="E5" s="7"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="7"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
+      <c r="G5" s="6"/>
+    </row>
+    <row r="6" spans="1:7" ht="20" customHeight="1">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
       <c r="C6" s="7"/>
       <c r="D6" s="8"/>
-      <c r="E6" s="7"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="7"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" ht="20" customHeight="1">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
       <c r="C7" s="7"/>
       <c r="D7" s="8"/>
-      <c r="E7" s="7"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="7"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
+      <c r="G7" s="6"/>
+    </row>
+    <row r="8" spans="1:7" ht="20" customHeight="1">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
       <c r="C8" s="7"/>
       <c r="D8" s="8"/>
-      <c r="E8" s="7"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="7"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
+      <c r="G8" s="6"/>
+    </row>
+    <row r="9" spans="1:7" ht="20" customHeight="1">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
       <c r="C9" s="7"/>
       <c r="D9" s="8"/>
-      <c r="E9" s="7"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="7"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" ht="20" customHeight="1">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="7"/>
       <c r="D10" s="8"/>
-      <c r="E10" s="7"/>
+      <c r="E10" s="6"/>
       <c r="F10" s="7"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" ht="20" customHeight="1">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
       <c r="C11" s="7"/>
       <c r="D11" s="8"/>
-      <c r="E11" s="7"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="7"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
+      <c r="G11" s="6"/>
+    </row>
+    <row r="12" spans="1:7" ht="20" customHeight="1">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
       <c r="C12" s="7"/>
       <c r="D12" s="8"/>
-      <c r="E12" s="7"/>
+      <c r="E12" s="10"/>
       <c r="F12" s="7"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
+      <c r="G12" s="6"/>
+    </row>
+    <row r="13" spans="1:7" ht="20" customHeight="1">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
       <c r="C13" s="7"/>
       <c r="D13" s="8"/>
-      <c r="E13" s="7"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="7"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
+      <c r="G13" s="6"/>
+    </row>
+    <row r="14" spans="1:7" ht="20" customHeight="1">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
       <c r="C14" s="7"/>
       <c r="D14" s="8"/>
-      <c r="E14" s="7"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="7"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" ht="20" customHeight="1">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
       <c r="C15" s="7"/>
       <c r="D15" s="8"/>
-      <c r="E15" s="7"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="7"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
+      <c r="G15" s="6"/>
+    </row>
+    <row r="16" spans="1:7" ht="20" customHeight="1">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
       <c r="C16" s="7"/>
       <c r="D16" s="8"/>
-      <c r="E16" s="7"/>
+      <c r="E16" s="6"/>
       <c r="F16" s="7"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" ht="20" customHeight="1">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
       <c r="C17" s="7"/>
       <c r="D17" s="8"/>
-      <c r="E17" s="7"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="7"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" ht="20" customHeight="1">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="7"/>
       <c r="D18" s="8"/>
-      <c r="E18" s="7"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="7"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" ht="20" customHeight="1">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="7"/>
       <c r="D19" s="8"/>
-      <c r="E19" s="7"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="7"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
+      <c r="G19" s="6"/>
+    </row>
+    <row r="20" spans="1:7" ht="20" customHeight="1">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="7"/>
       <c r="D20" s="8"/>
-      <c r="E20" s="7"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="7"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
+      <c r="G20" s="6"/>
+    </row>
+    <row r="21" spans="1:7" ht="20" customHeight="1">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
       <c r="C21" s="7"/>
       <c r="D21" s="8"/>
-      <c r="E21" s="7"/>
+      <c r="E21" s="6"/>
       <c r="F21" s="7"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-    </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C24" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="10">
-        <f>SUM(D2:D23)</f>
-      </c>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" ht="20" customHeight="1">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:7" ht="20" customHeight="1">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="C24" s="3"/>
+      <c r="D24" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="B10:B23">
-      <formula1>"交通,住宿,餐費,其他"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="B2:B23">
+  <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="B2:B23" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"交通,住宿,餐費,其他"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>